<commit_message>
fix superman and prep functions
</commit_message>
<xml_diff>
--- a/data-raw/superman/superman_raw.xlsx
+++ b/data-raw/superman/superman_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/docs/psych350data/data-raw/superman/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEF23DA-2369-AD48-B011-4D5ED3D69ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7517E50E-C40D-5245-AB6D-25568C60C166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="27600" windowHeight="18980" xr2:uid="{95E33088-5C19-2643-92D7-A985F3F12B6C}"/>
+    <workbookView xWindow="13480" yWindow="660" windowWidth="16020" windowHeight="18980" xr2:uid="{95E33088-5C19-2643-92D7-A985F3F12B6C}"/>
   </bookViews>
   <sheets>
     <sheet name="superman" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t>type</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>media</t>
+  </si>
+  <si>
+    <t>rt_critics_count</t>
+  </si>
+  <si>
+    <t>rt_audience_count</t>
   </si>
 </sst>
 </file>
@@ -1034,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11057603-1603-0F48-BF56-974BB2478A86}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -1047,10 +1053,12 @@
     <col min="8" max="8" width="10.83203125" style="1"/>
     <col min="9" max="9" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="1"/>
+    <col min="11" max="13" width="10.83203125" style="1"/>
+    <col min="14" max="14" width="11.5" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1085,16 +1093,22 @@
         <v>41</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1129,16 +1143,22 @@
         <v>83</v>
       </c>
       <c r="L2" s="1">
+        <v>484</v>
+      </c>
+      <c r="M2" s="1">
         <v>90</v>
       </c>
-      <c r="M2" s="1">
+      <c r="N2" s="1">
+        <v>25000</v>
+      </c>
+      <c r="O2" s="1">
         <v>1105511</v>
       </c>
-      <c r="N2" s="1">
+      <c r="P2" s="1">
         <v>3.9</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:16">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1173,16 +1193,22 @@
         <v>88</v>
       </c>
       <c r="L3" s="1">
+        <v>121</v>
+      </c>
+      <c r="M3" s="1">
         <v>86</v>
       </c>
-      <c r="M3" s="1">
+      <c r="N3" s="1">
+        <v>250000</v>
+      </c>
+      <c r="O3" s="1">
         <v>99115</v>
       </c>
-      <c r="N3" s="1">
+      <c r="P3" s="1">
         <v>3.7</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:16">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1217,10 +1243,16 @@
         <v>78</v>
       </c>
       <c r="L4" s="1">
+        <v>111</v>
+      </c>
+      <c r="M4" s="1">
         <v>72</v>
       </c>
+      <c r="N4" s="1">
+        <v>2500</v>
+      </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:16">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1255,16 +1287,22 @@
         <v>72</v>
       </c>
       <c r="L5" s="1">
+        <v>290</v>
+      </c>
+      <c r="M5" s="1">
         <v>60</v>
       </c>
-      <c r="M5" s="1">
+      <c r="N5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="O5" s="1">
         <v>26076</v>
       </c>
-      <c r="N5" s="1">
+      <c r="P5" s="1">
         <v>2.7</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:16">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1296,16 +1334,22 @@
         <v>9877</v>
       </c>
       <c r="L6" s="1">
+        <v>7</v>
+      </c>
+      <c r="M6" s="1">
         <v>79</v>
       </c>
-      <c r="M6" s="1">
+      <c r="N6" s="1">
+        <v>250</v>
+      </c>
+      <c r="O6" s="1">
         <v>744</v>
       </c>
-      <c r="N6" s="1">
+      <c r="P6" s="1">
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:16">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1340,16 +1384,22 @@
         <v>57</v>
       </c>
       <c r="L7" s="1">
+        <v>340</v>
+      </c>
+      <c r="M7" s="1">
         <v>75</v>
       </c>
-      <c r="M7" s="1">
+      <c r="N7" s="1">
+        <v>250000</v>
+      </c>
+      <c r="O7" s="1">
         <v>204463</v>
       </c>
-      <c r="N7" s="1">
+      <c r="P7" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:16">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1384,10 +1434,16 @@
         <v>83</v>
       </c>
       <c r="L8" s="1">
+        <v>484</v>
+      </c>
+      <c r="M8" s="1">
         <v>90</v>
       </c>
+      <c r="N8" s="1">
+        <v>25000</v>
+      </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:16">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1422,10 +1478,16 @@
         <v>88</v>
       </c>
       <c r="L9" s="1">
+        <v>55</v>
+      </c>
+      <c r="M9" s="1">
         <v>84</v>
       </c>
+      <c r="N9" s="1">
+        <v>1000</v>
+      </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:16">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1460,10 +1522,16 @@
         <v>86</v>
       </c>
       <c r="L10" s="1">
+        <v>20</v>
+      </c>
+      <c r="M10" s="1">
         <v>86</v>
       </c>
+      <c r="N10" s="1">
+        <v>100</v>
+      </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:16">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1486,7 +1554,7 @@
         <v>1.83</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:16">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>

</xml_diff>